<commit_message>
deploy: Shenzhen Synthetic Biology Infrastructure
</commit_message>
<xml_diff>
--- a/sdl-data.xlsx
+++ b/sdl-data.xlsx
@@ -9337,6 +9337,87 @@
         </is>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">szsynbio</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shenzhen Synthetic Biology Infrastructure</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAS SIAT</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shenzhen</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">China</t>
+        </is>
+      </c>
+      <c r="F114">
+        <v>22.74</v>
+      </c>
+      <c r="G114">
+        <v>113.92</v>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">national</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">biology</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">operational</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">multi-technique</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">strong</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">national facility</t>
+        </is>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">National major RI</t>
+        </is>
+      </c>
+      <c r="P114">
+        <v>2023</v>
+      </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://infrasynbio.siat.ac.cn/en</t>
+        </is>
+      </c>
+      <c r="R114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.siat.ac.cn/cxpt/202412/t20241214_7458457.html ; https://www.siat.ac.cn/symt/202604/t20260416_8186608.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -9357,7 +9438,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">112 initiatives across 15 countries</t>
+          <t xml:space="preserve">113 initiatives across 15 countries</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
deploy: ZJU iBioFoundry + iChemFoundry
</commit_message>
<xml_diff>
--- a/sdl-data.xlsx
+++ b/sdl-data.xlsx
@@ -9418,6 +9418,87 @@
         </is>
       </c>
     </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">zju-bmi</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZJU iBioFoundry + iChemFoundry</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Zhejiang University Hangzhou Innovation Center</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hangzhou</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">China</t>
+        </is>
+      </c>
+      <c r="F115">
+        <v>30.21</v>
+      </c>
+      <c r="G115">
+        <v>120.25</v>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">academic</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cross-domain</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">operational</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">multi-technique</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">strong</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">300+ instruments · 14,000 m²</t>
+        </is>
+      </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZJU + Hangzhou</t>
+        </is>
+      </c>
+      <c r="P115">
+        <v>2020</v>
+      </c>
+      <c r="Q115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://hic.zju.edu.cn/ibct/58279/list.htm</t>
+        </is>
+      </c>
+      <c r="R115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://hic.zju.edu.cn/ibct/58279/list.htm ; http://hic.zju.edu.cn/82840/list.htm</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -9438,7 +9519,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">113 initiatives across 15 countries</t>
+          <t xml:space="preserve">114 initiatives across 15 countries</t>
         </is>
       </c>
     </row>

</xml_diff>